<commit_message>
Last test of reproducible theta model
</commit_message>
<xml_diff>
--- a/parameters/neurons_parameters.xlsx
+++ b/parameters/neurons_parameters.xlsx
@@ -634,7 +634,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.62"/>
@@ -1641,7 +1641,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="11.11"/>
@@ -2645,7 +2645,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="11.62"/>
@@ -4138,7 +4138,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="26.64"/>
@@ -5619,7 +5619,7 @@
         <v>83</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E37" s="3" t="n">
         <v>1</v>
@@ -5629,7 +5629,7 @@
       </c>
       <c r="G37" s="3" t="n">
         <f aca="false">ROUND(F37*0.0025,0)*D37</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>59</v>

</xml_diff>

<commit_message>
Work on units model
</commit_message>
<xml_diff>
--- a/parameters/neurons_parameters.xlsx
+++ b/parameters/neurons_parameters.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="127">
   <si>
     <t xml:space="preserve">neurons</t>
   </si>
@@ -269,6 +269,9 @@
   </si>
   <si>
     <t xml:space="preserve">Simulated_Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delta_eta</t>
   </si>
   <si>
     <t xml:space="preserve">Axo-Axonic</t>
@@ -415,6 +418,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -435,6 +439,7 @@
       <sz val="10"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -479,7 +484,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -505,6 +510,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -632,7 +641,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.62"/>
@@ -1639,7 +1648,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="11.11"/>
@@ -2643,7 +2652,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="11.62"/>
@@ -4135,8 +4144,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:P42"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="26.64"/>
@@ -4197,16 +4206,19 @@
       <c r="O1" s="3" t="s">
         <v>68</v>
       </c>
+      <c r="P1" s="7" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>1</v>
@@ -4241,6 +4253,9 @@
       </c>
       <c r="N2" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P2" s="0" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4248,10 +4263,10 @@
         <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>83</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>1</v>
@@ -4286,10 +4301,10 @@
         <v>13</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>1</v>
@@ -4324,10 +4339,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D5" s="3" t="n">
         <v>1</v>
@@ -4362,6 +4377,9 @@
       </c>
       <c r="N5" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P5" s="0" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4369,10 +4387,10 @@
         <v>17</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>1</v>
@@ -4407,10 +4425,10 @@
         <v>18</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D7" s="3" t="n">
         <v>1</v>
@@ -4445,6 +4463,9 @@
       </c>
       <c r="N7" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P7" s="0" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4452,10 +4473,10 @@
         <v>21</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>1</v>
@@ -4489,6 +4510,9 @@
       </c>
       <c r="N8" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P8" s="0" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4496,10 +4520,10 @@
         <v>23</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D9" s="3" t="n">
         <v>0</v>
@@ -4535,10 +4559,10 @@
         <v>24</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D10" s="3" t="n">
         <v>1</v>
@@ -4572,6 +4596,9 @@
       </c>
       <c r="N10" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P10" s="0" t="n">
+        <v>80</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4579,10 +4606,10 @@
         <v>26</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D11" s="3" t="n">
         <v>1</v>
@@ -4617,10 +4644,10 @@
         <v>27</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D12" s="3" t="n">
         <v>1</v>
@@ -4656,10 +4683,10 @@
         <v>28</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>1</v>
@@ -4695,10 +4722,10 @@
         <v>29</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>1</v>
@@ -4733,10 +4760,10 @@
         <v>30</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D15" s="3" t="n">
         <v>1</v>
@@ -4771,10 +4798,10 @@
         <v>31</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D16" s="3" t="n">
         <v>1</v>
@@ -4808,6 +4835,9 @@
       </c>
       <c r="N16" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P16" s="0" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4815,10 +4845,10 @@
         <v>33</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>1</v>
@@ -4854,10 +4884,10 @@
         <v>34</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>1</v>
@@ -4899,10 +4929,10 @@
         <v>36</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D19" s="3" t="n">
         <v>0</v>
@@ -4938,10 +4968,10 @@
         <v>37</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D20" s="3" t="n">
         <v>1</v>
@@ -4976,10 +5006,10 @@
         <v>38</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>0</v>
@@ -5015,10 +5045,10 @@
         <v>39</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>1</v>
@@ -5054,10 +5084,10 @@
         <v>40</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>1</v>
@@ -5092,10 +5122,10 @@
         <v>41</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>1</v>
@@ -5130,10 +5160,10 @@
         <v>42</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>1</v>
@@ -5169,10 +5199,10 @@
         <v>43</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D26" s="3" t="n">
         <v>1</v>
@@ -5207,10 +5237,10 @@
         <v>44</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D27" s="3" t="n">
         <v>1</v>
@@ -5245,6 +5275,9 @@
       </c>
       <c r="N27" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P27" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5252,10 +5285,10 @@
         <v>47</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D28" s="3" t="n">
         <v>0</v>
@@ -5291,10 +5324,10 @@
         <v>48</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D29" s="3" t="n">
         <v>0</v>
@@ -5330,10 +5363,10 @@
         <v>49</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D30" s="3" t="n">
         <v>1</v>
@@ -5367,6 +5400,9 @@
       </c>
       <c r="N30" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P30" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5374,10 +5410,10 @@
         <v>52</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D31" s="3" t="n">
         <v>1</v>
@@ -5413,10 +5449,10 @@
         <v>53</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D32" s="3" t="n">
         <v>1</v>
@@ -5452,10 +5488,10 @@
         <v>54</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D33" s="3" t="n">
         <v>1</v>
@@ -5489,6 +5525,9 @@
       </c>
       <c r="N33" s="3" t="n">
         <v>0</v>
+      </c>
+      <c r="P33" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5496,10 +5535,10 @@
         <v>55</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D34" s="3" t="n">
         <v>1</v>
@@ -5537,7 +5576,7 @@
         <v>56</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D35" s="3" t="n">
         <v>1</v>
@@ -5573,10 +5612,10 @@
         <v>57</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D36" s="3" t="n">
         <v>1</v>
@@ -5611,10 +5650,10 @@
         <v>58</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D37" s="3" t="n">
         <v>0</v>
@@ -5656,10 +5695,10 @@
         <v>61</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D38" s="3" t="n">
         <v>0</v>
@@ -5692,13 +5731,13 @@
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>1</v>
@@ -5736,13 +5775,13 @@
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>122</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="D40" s="3" t="n">
         <v>1</v>
@@ -5783,10 +5822,10 @@
         <v>8</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D41" s="4" t="n">
         <v>1</v>
@@ -5827,10 +5866,10 @@
         <v>8</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D42" s="4" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Unit simulation need testing
</commit_message>
<xml_diff>
--- a/parameters/neurons_parameters.xlsx
+++ b/parameters/neurons_parameters.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="127">
   <si>
     <t xml:space="preserve">neurons</t>
   </si>
@@ -641,7 +641,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.62"/>
@@ -1648,7 +1648,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="11.11"/>
@@ -2652,7 +2652,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="11.62"/>
@@ -4145,7 +4145,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="26.64"/>
@@ -5276,8 +5276,8 @@
       <c r="N27" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="P27" s="2" t="n">
-        <v>3</v>
+      <c r="P27" s="2" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5402,7 +5402,7 @@
         <v>0</v>
       </c>
       <c r="P30" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5527,7 +5527,7 @@
         <v>0</v>
       </c>
       <c r="P33" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Work on stable work of the model
</commit_message>
<xml_diff>
--- a/parameters/neurons_parameters.xlsx
+++ b/parameters/neurons_parameters.xlsx
@@ -641,7 +641,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.62"/>
@@ -1648,7 +1648,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="3" width="11.11"/>
@@ -2652,7 +2652,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="11.62"/>
@@ -4145,7 +4145,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="26.64"/>
@@ -4923,6 +4923,9 @@
       <c r="N18" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="P18" s="0" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">

</xml_diff>

<commit_message>
Start to work with big local model
</commit_message>
<xml_diff>
--- a/parameters/neurons_parameters.xlsx
+++ b/parameters/neurons_parameters.xlsx
@@ -796,7 +796,7 @@
       </c>
       <c r="O2" s="3"/>
       <c r="P2" s="2" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -927,7 +927,7 @@
       </c>
       <c r="O5" s="3"/>
       <c r="P5" s="2" t="n">
-        <v>25</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1017,7 +1017,7 @@
       </c>
       <c r="O7" s="3"/>
       <c r="P7" s="2" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1112,6 +1112,9 @@
         <v>0</v>
       </c>
       <c r="O9" s="6"/>
+      <c r="P9" s="7" t="n">
+        <v>50</v>
+      </c>
       <c r="Q9" s="8" t="s">
         <v>43</v>
       </c>
@@ -1892,7 +1895,7 @@
       </c>
       <c r="O27" s="3"/>
       <c r="P27" s="2" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2024,7 +2027,7 @@
       </c>
       <c r="O30" s="3"/>
       <c r="P30" s="2" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2156,7 +2159,7 @@
       </c>
       <c r="O33" s="3"/>
       <c r="P33" s="2" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2203,6 +2206,9 @@
         <v>0</v>
       </c>
       <c r="O34" s="6"/>
+      <c r="P34" s="7" t="n">
+        <v>50</v>
+      </c>
       <c r="Q34" s="9" t="s">
         <v>104</v>
       </c>
@@ -2334,6 +2340,9 @@
         <v>0</v>
       </c>
       <c r="O37" s="3"/>
+      <c r="P37" s="0" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">

</xml_diff>

<commit_message>
Added: * Integration error * Pyramidal cells
</commit_message>
<xml_diff>
--- a/parameters/neurons_parameters.xlsx
+++ b/parameters/neurons_parameters.xlsx
@@ -76,18 +76,36 @@
     <t xml:space="preserve">Источник</t>
   </si>
   <si>
+    <t xml:space="preserve">CA1 Pyramidal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pyramidal (deep)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">simulated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pyramidal (superficial)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.14</t>
+  </si>
+  <si>
     <t xml:space="preserve">CA1 Axo-Axonic</t>
   </si>
   <si>
     <t xml:space="preserve">Axo-Axonic</t>
   </si>
   <si>
-    <t xml:space="preserve">simulated</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0</t>
-  </si>
-  <si>
     <t xml:space="preserve">0.3</t>
   </si>
   <si>
@@ -139,9 +157,6 @@
     <t xml:space="preserve">Bistratified</t>
   </si>
   <si>
-    <t xml:space="preserve">3.14</t>
-  </si>
-  <si>
     <t xml:space="preserve">CA1 Hippocampo-subicular Projecting ENK+</t>
   </si>
   <si>
@@ -376,12 +391,6 @@
     <t xml:space="preserve">1.4</t>
   </si>
   <si>
-    <t xml:space="preserve">0.25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.5</t>
-  </si>
-  <si>
     <t xml:space="preserve">EC LIII Pyramidal</t>
   </si>
   <si>
@@ -389,15 +398,6 @@
   </si>
   <si>
     <t xml:space="preserve">1.5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CA1 Pyramidal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pyramidal (deep)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pyramidal (superficial)</t>
   </si>
   <si>
     <t xml:space="preserve">neurons</t>
@@ -434,7 +434,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -455,6 +455,11 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -512,7 +517,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -537,19 +542,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -557,7 +554,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -684,7 +681,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:Q42"/>
+  <dimension ref="A1:Q44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
@@ -746,41 +743,40 @@
       <c r="P1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="0" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="3" t="n">
+      <c r="C2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="4" t="n">
         <v>1</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>312</v>
-      </c>
-      <c r="G2" s="3" t="n">
-        <f aca="false">ROUND(F2*0.0025,0)*D2</f>
-        <v>1</v>
-      </c>
-      <c r="H2" s="3" t="s">
+      <c r="F2" s="4" t="n">
+        <v>160000</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="3" t="n">
-        <v>29</v>
+      <c r="J2" s="4" t="s">
+        <v>22</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>8</v>
@@ -795,37 +791,38 @@
         <v>0</v>
       </c>
       <c r="O2" s="3"/>
-      <c r="P2" s="2" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>160000</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="3" t="n">
-        <v>203</v>
-      </c>
-      <c r="G3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="3"/>
       <c r="K3" s="3" t="n">
         <v>8</v>
       </c>
@@ -842,10 +839,10 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>19</v>
@@ -857,16 +854,21 @@
         <v>1</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>793</v>
+        <v>312</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3"/>
+        <f aca="false">ROUND(F4*0.0025,0)*D4</f>
+        <v>1</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="I4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" s="3"/>
+        <v>27</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>29</v>
+      </c>
       <c r="K4" s="3" t="n">
         <v>8</v>
       </c>
@@ -880,13 +882,16 @@
         <v>0</v>
       </c>
       <c r="O4" s="3"/>
+      <c r="P4" s="2" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>19</v>
@@ -898,21 +903,16 @@
         <v>1</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>336</v>
+        <v>203</v>
       </c>
       <c r="G5" s="3" t="n">
-        <f aca="false">ROUND(F5*0.0025,0)*D5</f>
-        <v>1</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>28</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H5" s="3"/>
       <c r="I5" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>29</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="J5" s="3"/>
       <c r="K5" s="3" t="n">
         <v>8</v>
       </c>
@@ -926,9 +926,6 @@
         <v>0</v>
       </c>
       <c r="O5" s="3"/>
-      <c r="P5" s="2" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
@@ -947,14 +944,14 @@
         <v>1</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>333</v>
+        <v>793</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J6" s="3"/>
       <c r="K6" s="3" t="n">
@@ -988,7 +985,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>395</v>
+        <v>336</v>
       </c>
       <c r="G7" s="3" t="n">
         <f aca="false">ROUND(F7*0.0025,0)*D7</f>
@@ -998,7 +995,7 @@
         <v>34</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>35</v>
@@ -1037,94 +1034,85 @@
         <v>1</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>804</v>
+        <v>333</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="3"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="I8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J8" s="3" t="n">
-        <v>27</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L8" s="3" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M8" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N8" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="3"/>
-      <c r="P8" s="2" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
+      <c r="B9" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>395</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <f aca="false">ROUND(F9*0.0025,0)*D9</f>
+        <v>1</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>118</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="6" t="s">
+      <c r="I9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="I9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M9" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="N9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="6"/>
-      <c r="P9" s="7" t="n">
+      <c r="K9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="3"/>
+      <c r="P9" s="2" t="n">
         <v>50</v>
-      </c>
-      <c r="Q9" s="8" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>19</v>
@@ -1136,19 +1124,19 @@
         <v>1</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>778</v>
+        <v>804</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>46</v>
+        <v>27</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>27</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>8</v>
@@ -1164,49 +1152,59 @@
       </c>
       <c r="O10" s="3"/>
       <c r="P10" s="2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>118</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4"/>
+      <c r="P11" s="2" t="n">
         <v>50</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B11" s="3" t="s">
+      <c r="Q11" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="3" t="n">
-        <v>837</v>
-      </c>
-      <c r="G11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L11" s="3" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M11" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="3"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
@@ -1222,20 +1220,23 @@
         <v>1</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>171</v>
+        <v>778</v>
       </c>
       <c r="G12" s="3" t="n">
-        <f aca="false">ROUND(F12*0.0025,0)*D12</f>
-        <v>0</v>
-      </c>
-      <c r="H12" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="I12" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J12" s="3"/>
+        <v>27</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>51</v>
+      </c>
       <c r="K12" s="3" t="n">
         <v>8</v>
       </c>
@@ -1249,13 +1250,16 @@
         <v>0</v>
       </c>
       <c r="O12" s="3"/>
+      <c r="P12" s="2" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>19</v>
@@ -1264,18 +1268,17 @@
         <v>1</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>136</v>
+        <v>837</v>
       </c>
       <c r="G13" s="3" t="n">
-        <f aca="false">ROUND(F13*0.0025,0)*D13</f>
         <v>0</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J13" s="3"/>
       <c r="K13" s="3" t="n">
@@ -1294,10 +1297,10 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>19</v>
@@ -1309,14 +1312,15 @@
         <v>0</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>1010</v>
+        <v>171</v>
       </c>
       <c r="G14" s="3" t="n">
+        <f aca="false">ROUND(F14*0.0025,0)*D14</f>
         <v>0</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J14" s="3"/>
       <c r="K14" s="3" t="n">
@@ -1335,10 +1339,10 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>19</v>
@@ -1347,17 +1351,18 @@
         <v>1</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>658</v>
+        <v>136</v>
       </c>
       <c r="G15" s="3" t="n">
+        <f aca="false">ROUND(F15*0.0025,0)*D15</f>
         <v>0</v>
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J15" s="3"/>
       <c r="K15" s="3" t="n">
@@ -1376,10 +1381,10 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>19</v>
@@ -1388,23 +1393,19 @@
         <v>1</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>1114</v>
+        <v>1010</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>20</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H16" s="3"/>
       <c r="I16" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>59</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="J16" s="3"/>
       <c r="K16" s="3" t="n">
         <v>8</v>
       </c>
@@ -1418,87 +1419,78 @@
         <v>0</v>
       </c>
       <c r="O16" s="3"/>
-      <c r="P16" s="2" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="6" t="n">
-        <v>96</v>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="J17" s="6"/>
-      <c r="K17" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L17" s="6" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M17" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="6"/>
-      <c r="Q17" s="8" t="s">
-        <v>62</v>
-      </c>
+      <c r="C17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>658</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="3"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>1114</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J18" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>521</v>
-      </c>
-      <c r="G18" s="3" t="n">
-        <f aca="false">ROUND(F18*0.0025,0)*D18</f>
-        <v>1</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>65</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>8</v>
@@ -1514,50 +1506,54 @@
       </c>
       <c r="O18" s="3"/>
       <c r="P18" s="2" t="n">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>96</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J19" s="4"/>
+      <c r="K19" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L19" s="4" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M19" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4"/>
+      <c r="Q19" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <f aca="false">ROUND(F19*0.0025,0)*D19</f>
-        <v>0</v>
-      </c>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L19" s="3" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M19" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
@@ -1576,16 +1572,21 @@
         <v>1</v>
       </c>
       <c r="F20" s="3" t="n">
-        <v>574</v>
+        <v>521</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" s="3"/>
+        <f aca="false">ROUND(F20*0.0025,0)*D20</f>
+        <v>1</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>24</v>
+      </c>
       <c r="I20" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J20" s="3"/>
+        <v>27</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>70</v>
+      </c>
       <c r="K20" s="3" t="n">
         <v>8</v>
       </c>
@@ -1599,25 +1600,28 @@
         <v>0</v>
       </c>
       <c r="O20" s="3"/>
+      <c r="P20" s="2" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="3" t="n">
         <v>70</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="3" t="n">
-        <v>73</v>
       </c>
       <c r="G21" s="3" t="n">
         <f aca="false">ROUND(F21*0.0025,0)*D21</f>
@@ -1625,7 +1629,7 @@
       </c>
       <c r="H21" s="3"/>
       <c r="I21" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="3" t="n">
@@ -1644,10 +1648,10 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>19</v>
@@ -1656,18 +1660,17 @@
         <v>1</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F22" s="3" t="n">
-        <v>171</v>
+        <v>574</v>
       </c>
       <c r="G22" s="3" t="n">
-        <f aca="false">ROUND(F22*0.0025,0)*D22</f>
         <v>0</v>
       </c>
       <c r="H22" s="3"/>
       <c r="I22" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="3" t="n">
@@ -1686,29 +1689,30 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>607</v>
+        <v>73</v>
       </c>
       <c r="G23" s="3" t="n">
+        <f aca="false">ROUND(F23*0.0025,0)*D23</f>
         <v>0</v>
       </c>
       <c r="H23" s="3"/>
       <c r="I23" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J23" s="3"/>
       <c r="K23" s="3" t="n">
@@ -1727,10 +1731,10 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>19</v>
@@ -1739,17 +1743,18 @@
         <v>1</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" s="3" t="n">
-        <v>340</v>
+        <v>171</v>
       </c>
       <c r="G24" s="3" t="n">
+        <f aca="false">ROUND(F24*0.0025,0)*D24</f>
         <v>0</v>
       </c>
       <c r="H24" s="3"/>
       <c r="I24" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J24" s="3"/>
       <c r="K24" s="3" t="n">
@@ -1768,10 +1773,10 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>19</v>
@@ -1780,18 +1785,17 @@
         <v>1</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" s="3" t="n">
-        <v>191</v>
+        <v>607</v>
       </c>
       <c r="G25" s="3" t="n">
-        <f aca="false">ROUND(F25*0.0025,0)*D25</f>
         <v>0</v>
       </c>
       <c r="H25" s="3"/>
       <c r="I25" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J25" s="3"/>
       <c r="K25" s="3" t="n">
@@ -1810,10 +1814,10 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>19</v>
@@ -1825,14 +1829,14 @@
         <v>1</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>729</v>
+        <v>340</v>
       </c>
       <c r="G26" s="3" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="3"/>
       <c r="I26" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J26" s="3"/>
       <c r="K26" s="3" t="n">
@@ -1850,12 +1854,12 @@
       <c r="O26" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B27" s="4" t="s">
+      <c r="A27" s="3" t="s">
         <v>83</v>
       </c>
+      <c r="B27" s="3" t="s">
+        <v>84</v>
+      </c>
       <c r="C27" s="4" t="s">
         <v>19</v>
       </c>
@@ -1863,24 +1867,20 @@
         <v>1</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>463</v>
+        <v>191</v>
       </c>
       <c r="G27" s="3" t="n">
         <f aca="false">ROUND(F27*0.0025,0)*D27</f>
-        <v>1</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>84</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H27" s="3"/>
       <c r="I27" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J27" s="3" t="s">
-        <v>85</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="J27" s="3"/>
       <c r="K27" s="3" t="n">
         <v>8</v>
       </c>
@@ -1894,36 +1894,32 @@
         <v>0</v>
       </c>
       <c r="O27" s="3"/>
-      <c r="P27" s="2" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B28" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B28" s="3" t="s">
-        <v>87</v>
-      </c>
       <c r="C28" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F28" s="3" t="n">
-        <v>22</v>
+        <v>729</v>
       </c>
       <c r="G28" s="3" t="n">
-        <f aca="false">ROUND(F28*0.0025,0)*D28</f>
         <v>0</v>
       </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J28" s="3"/>
       <c r="K28" s="3" t="n">
@@ -1941,33 +1937,37 @@
       <c r="O28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
+      <c r="A29" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="B29" s="3" t="s">
-        <v>89</v>
-      </c>
       <c r="C29" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E29" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>9</v>
+        <v>463</v>
       </c>
       <c r="G29" s="3" t="n">
         <f aca="false">ROUND(F29*0.0025,0)*D29</f>
-        <v>0</v>
-      </c>
-      <c r="H29" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>89</v>
+      </c>
       <c r="I29" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J29" s="3"/>
+        <v>27</v>
+      </c>
+      <c r="J29" s="3" t="s">
+        <v>90</v>
+      </c>
       <c r="K29" s="3" t="n">
         <v>8</v>
       </c>
@@ -1981,38 +1981,38 @@
         <v>0</v>
       </c>
       <c r="O29" s="3"/>
+      <c r="P29" s="2" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" s="3" t="n">
-        <v>698</v>
+        <v>22</v>
       </c>
       <c r="G30" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>92</v>
-      </c>
+        <f aca="false">ROUND(F30*0.0025,0)*D30</f>
+        <v>0</v>
+      </c>
+      <c r="H30" s="3"/>
       <c r="I30" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J30" s="3" t="s">
-        <v>93</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="J30" s="3"/>
       <c r="K30" s="3" t="n">
         <v>8</v>
       </c>
@@ -2026,28 +2026,25 @@
         <v>0</v>
       </c>
       <c r="O30" s="3"/>
-      <c r="P30" s="2" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B31" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B31" s="3" t="s">
-        <v>95</v>
-      </c>
       <c r="C31" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D31" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E31" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>128</v>
+        <v>9</v>
       </c>
       <c r="G31" s="3" t="n">
         <f aca="false">ROUND(F31*0.0025,0)*D31</f>
@@ -2055,7 +2052,7 @@
       </c>
       <c r="H31" s="3"/>
       <c r="I31" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J31" s="3"/>
       <c r="K31" s="3" t="n">
@@ -2074,32 +2071,35 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B32" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="C32" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>698</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D32" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E32" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="3" t="n">
-        <v>93</v>
-      </c>
-      <c r="G32" s="3" t="n">
-        <f aca="false">ROUND(F32*0.0025,0)*D32</f>
-        <v>0</v>
-      </c>
-      <c r="H32" s="3"/>
       <c r="I32" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J32" s="3"/>
+        <v>27</v>
+      </c>
+      <c r="J32" s="3" t="s">
+        <v>98</v>
+      </c>
       <c r="K32" s="3" t="n">
         <v>8</v>
       </c>
@@ -2113,13 +2113,16 @@
         <v>0</v>
       </c>
       <c r="O32" s="3"/>
+      <c r="P32" s="2" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>19</v>
@@ -2128,205 +2131,203 @@
         <v>1</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>171</v>
+        <v>128</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>92</v>
-      </c>
+        <f aca="false">ROUND(F33*0.0025,0)*D33</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="3"/>
       <c r="I33" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J33" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L33" s="3" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M33" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="3" t="n">
         <v>93</v>
       </c>
-      <c r="K33" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L33" s="3" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M33" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" s="3"/>
-      <c r="P33" s="2" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="34" s="7" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="E34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="6" t="n">
-        <v>986</v>
-      </c>
-      <c r="G34" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="I34" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="J34" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="K34" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L34" s="6" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M34" s="6" t="n">
-        <v>100</v>
-      </c>
-      <c r="N34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O34" s="6"/>
-      <c r="P34" s="7" t="n">
-        <v>50</v>
-      </c>
-      <c r="Q34" s="9" t="s">
-        <v>104</v>
-      </c>
+      <c r="G34" s="3" t="n">
+        <f aca="false">ROUND(F34*0.0025,0)*D34</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L34" s="3" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M34" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="3"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>171</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="I35" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="K35" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L35" s="3" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M35" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O35" s="3"/>
+      <c r="P35" s="2" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B35" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D35" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="3" t="n">
-        <v>84</v>
-      </c>
-      <c r="G35" s="3" t="n">
-        <f aca="false">ROUND(F35*0.0025,0)*D35</f>
-        <v>0</v>
-      </c>
-      <c r="H35" s="3"/>
-      <c r="I35" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J35" s="3"/>
-      <c r="K35" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L35" s="3" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M35" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O35" s="3"/>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="B36" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="C36" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>986</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="C36" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D36" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E36" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="3" t="n">
-        <v>313</v>
-      </c>
-      <c r="G36" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="3"/>
-      <c r="I36" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J36" s="3"/>
-      <c r="K36" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L36" s="3" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M36" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N36" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O36" s="3"/>
+      <c r="I36" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="N36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O36" s="4"/>
+      <c r="P36" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q36" s="5" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D37" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E37" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F37" s="3" t="n">
-        <v>401</v>
+        <v>84</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>110</v>
-      </c>
+        <f aca="false">ROUND(F37*0.0025,0)*D37</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="3"/>
       <c r="I37" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>103</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="J37" s="3"/>
       <c r="K37" s="3" t="n">
         <v>8</v>
       </c>
@@ -2340,9 +2341,6 @@
         <v>0</v>
       </c>
       <c r="O37" s="3"/>
-      <c r="P37" s="0" t="n">
-        <v>50</v>
-      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
@@ -2355,21 +2353,20 @@
         <v>19</v>
       </c>
       <c r="D38" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E38" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F38" s="3" t="n">
-        <v>119</v>
+        <v>313</v>
       </c>
       <c r="G38" s="3" t="n">
-        <f aca="false">ROUND(F38*0.0025,0)*D38</f>
         <v>0</v>
       </c>
       <c r="H38" s="3"/>
       <c r="I38" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J38" s="3"/>
       <c r="K38" s="3" t="n">
@@ -2393,29 +2390,29 @@
       <c r="B39" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>401</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G39" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>116</v>
-      </c>
       <c r="I39" s="3" t="s">
-        <v>117</v>
+        <v>27</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="K39" s="3" t="n">
         <v>8</v>
@@ -2430,128 +2427,128 @@
         <v>0</v>
       </c>
       <c r="O39" s="3"/>
+      <c r="P39" s="2" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="3" t="n">
         <v>119</v>
       </c>
-      <c r="B40" s="3" t="s">
+      <c r="G40" s="3" t="n">
+        <f aca="false">ROUND(F40*0.0025,0)*D40</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L40" s="3" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M40" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O40" s="3"/>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="C41" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D40" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E40" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="I40" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="J40" s="3" t="s">
+      <c r="D41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="K40" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L40" s="3" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M40" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N40" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O40" s="3"/>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="I41" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="L41" s="3" t="n">
+        <v>-100000</v>
+      </c>
+      <c r="M41" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="N41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O41" s="3"/>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B42" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C41" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E41" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="4" t="n">
-        <v>160000</v>
-      </c>
-      <c r="G41" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H41" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I41" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="J41" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="K41" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="L41" s="3" t="n">
-        <v>-100000</v>
-      </c>
-      <c r="M41" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="N41" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O41" s="3"/>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="B42" s="4" t="s">
+      <c r="C42" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="J42" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C42" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="D42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E42" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="4" t="n">
-        <v>160000</v>
-      </c>
-      <c r="G42" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H42" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I42" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="J42" s="4" t="s">
-        <v>118</v>
-      </c>
       <c r="K42" s="3" t="n">
         <v>8</v>
       </c>
@@ -2565,11 +2562,33 @@
         <v>0</v>
       </c>
       <c r="O42" s="3"/>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="0"/>
+      <c r="B43" s="0"/>
+      <c r="C43" s="0"/>
+      <c r="D43" s="0"/>
+      <c r="E43" s="0"/>
+      <c r="F43" s="0"/>
+      <c r="G43" s="0"/>
+      <c r="H43" s="0"/>
+      <c r="I43" s="0"/>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0"/>
+      <c r="B44" s="0"/>
+      <c r="C44" s="0"/>
+      <c r="D44" s="0"/>
+      <c r="E44" s="0"/>
+      <c r="F44" s="0"/>
+      <c r="G44" s="0"/>
+      <c r="H44" s="0"/>
+      <c r="I44" s="0"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="Q9" r:id="rId1" display="http://www.ncbi.nlm.nih.gov/pubmed?term=PMID:%2018829959"/>
-    <hyperlink ref="Q17" r:id="rId2" display="https://www.jneurosci.org/content/30/5/1595.long"/>
+    <hyperlink ref="Q11" r:id="rId1" display="http://www.ncbi.nlm.nih.gov/pubmed?term=PMID:%2018829959"/>
+    <hyperlink ref="Q19" r:id="rId2" display="https://www.jneurosci.org/content/30/5/1595.long"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -2623,8 +2642,8 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
-        <v>122</v>
+      <c r="A2" s="8" t="s">
+        <v>17</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>1</v>
@@ -2644,7 +2663,7 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B3" s="3" t="n">
         <v>1</v>
@@ -2663,16 +2682,16 @@
         <v>20</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>29</v>
       </c>
-      <c r="I3" s="11"/>
+      <c r="I3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>1</v>
@@ -2689,14 +2708,14 @@
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H4" s="3"/>
-      <c r="I4" s="11"/>
+      <c r="I4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>1</v>
@@ -2713,14 +2732,14 @@
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H5" s="3"/>
-      <c r="I5" s="11"/>
+      <c r="I5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>1</v>
@@ -2736,19 +2755,19 @@
         <v>34</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="11"/>
+        <v>35</v>
+      </c>
+      <c r="I6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>1</v>
@@ -2765,14 +2784,14 @@
       </c>
       <c r="F7" s="3"/>
       <c r="G7" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H7" s="3"/>
-      <c r="I7" s="11"/>
+      <c r="I7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>1</v>
@@ -2788,19 +2807,19 @@
         <v>40</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="I8" s="11"/>
+        <v>41</v>
+      </c>
+      <c r="I8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>1</v>
@@ -2816,19 +2835,19 @@
         <v>80</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>27</v>
       </c>
-      <c r="I9" s="11"/>
+      <c r="I9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>0</v>
@@ -2845,14 +2864,14 @@
       </c>
       <c r="F10" s="3"/>
       <c r="G10" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H10" s="3"/>
-      <c r="I10" s="11"/>
+      <c r="I10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>1</v>
@@ -2868,19 +2887,19 @@
         <v>78</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="I11" s="11"/>
+        <v>51</v>
+      </c>
+      <c r="I11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>1</v>
@@ -2897,14 +2916,14 @@
       </c>
       <c r="F12" s="3"/>
       <c r="G12" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H12" s="3"/>
-      <c r="I12" s="11"/>
+      <c r="I12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>1</v>
@@ -2921,14 +2940,14 @@
       </c>
       <c r="F13" s="3"/>
       <c r="G13" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H13" s="3"/>
-      <c r="I13" s="11"/>
+      <c r="I13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>1</v>
@@ -2945,14 +2964,14 @@
       </c>
       <c r="F14" s="3"/>
       <c r="G14" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H14" s="3"/>
-      <c r="I14" s="11"/>
+      <c r="I14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>1</v>
@@ -2969,14 +2988,14 @@
       </c>
       <c r="F15" s="3"/>
       <c r="G15" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H15" s="3"/>
-      <c r="I15" s="11"/>
+      <c r="I15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>1</v>
@@ -2993,14 +3012,14 @@
       </c>
       <c r="F16" s="3"/>
       <c r="G16" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H16" s="3"/>
-      <c r="I16" s="11"/>
+      <c r="I16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>1</v>
@@ -3019,16 +3038,16 @@
         <v>20</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="I17" s="11"/>
+        <v>64</v>
+      </c>
+      <c r="I17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>1</v>
@@ -3045,14 +3064,14 @@
       </c>
       <c r="F18" s="3"/>
       <c r="G18" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H18" s="3"/>
-      <c r="I18" s="11"/>
+      <c r="I18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>1</v>
@@ -3068,19 +3087,19 @@
         <v>52</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="I19" s="11"/>
+        <v>70</v>
+      </c>
+      <c r="I19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>0</v>
@@ -3097,14 +3116,14 @@
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H20" s="3"/>
-      <c r="I20" s="11"/>
+      <c r="I20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>1</v>
@@ -3121,14 +3140,14 @@
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H21" s="3"/>
-      <c r="I21" s="11"/>
+      <c r="I21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>0</v>
@@ -3145,14 +3164,14 @@
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H22" s="3"/>
-      <c r="I22" s="11"/>
+      <c r="I22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>1</v>
@@ -3169,14 +3188,14 @@
       </c>
       <c r="F23" s="3"/>
       <c r="G23" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H23" s="3"/>
-      <c r="I23" s="11"/>
+      <c r="I23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>1</v>
@@ -3193,14 +3212,14 @@
       </c>
       <c r="F24" s="3"/>
       <c r="G24" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H24" s="3"/>
-      <c r="I24" s="11"/>
+      <c r="I24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>1</v>
@@ -3217,14 +3236,14 @@
       </c>
       <c r="F25" s="3"/>
       <c r="G25" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H25" s="3"/>
-      <c r="I25" s="11"/>
-    </row>
-    <row r="26" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I25" s="9"/>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>1</v>
@@ -3241,14 +3260,14 @@
       </c>
       <c r="F26" s="3"/>
       <c r="G26" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H26" s="3"/>
-      <c r="I26" s="11"/>
+      <c r="I26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>1</v>
@@ -3265,14 +3284,14 @@
       </c>
       <c r="F27" s="3"/>
       <c r="G27" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H27" s="3"/>
-      <c r="I27" s="11"/>
+      <c r="I27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="s">
-        <v>82</v>
+      <c r="A28" s="8" t="s">
+        <v>87</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>1</v>
@@ -3288,19 +3307,19 @@
         <v>46</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="I28" s="11"/>
+        <v>90</v>
+      </c>
+      <c r="I28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>0</v>
@@ -3317,14 +3336,14 @@
       </c>
       <c r="F29" s="3"/>
       <c r="G29" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H29" s="3"/>
-      <c r="I29" s="11"/>
+      <c r="I29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0</v>
@@ -3341,14 +3360,14 @@
       </c>
       <c r="F30" s="3"/>
       <c r="G30" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H30" s="3"/>
-      <c r="I30" s="11"/>
+      <c r="I30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>1</v>
@@ -3364,19 +3383,19 @@
         <v>70</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="I31" s="11"/>
+        <v>98</v>
+      </c>
+      <c r="I31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>1</v>
@@ -3393,14 +3412,14 @@
       </c>
       <c r="F32" s="3"/>
       <c r="G32" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H32" s="3"/>
-      <c r="I32" s="11"/>
-    </row>
-    <row r="33" s="2" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I32" s="9"/>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>1</v>
@@ -3417,14 +3436,14 @@
       </c>
       <c r="F33" s="3"/>
       <c r="G33" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H33" s="3"/>
-      <c r="I33" s="11"/>
+      <c r="I33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>1</v>
@@ -3440,19 +3459,19 @@
         <v>17</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="I34" s="11"/>
+        <v>98</v>
+      </c>
+      <c r="I34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="s">
-        <v>100</v>
+      <c r="A35" s="8" t="s">
+        <v>105</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>1</v>
@@ -3469,14 +3488,14 @@
       </c>
       <c r="F35" s="3"/>
       <c r="G35" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H35" s="3"/>
-      <c r="I35" s="11"/>
+      <c r="I35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>1</v>
@@ -3493,14 +3512,14 @@
       </c>
       <c r="F36" s="3"/>
       <c r="G36" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H36" s="3"/>
-      <c r="I36" s="11"/>
+      <c r="I36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>1</v>
@@ -3517,14 +3536,14 @@
       </c>
       <c r="F37" s="3"/>
       <c r="G37" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H37" s="3"/>
-      <c r="I37" s="11"/>
+      <c r="I37" s="9"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>1</v>
@@ -3540,19 +3559,19 @@
         <v>40</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="I38" s="11"/>
+      <c r="I38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>0</v>
@@ -3569,10 +3588,10 @@
       </c>
       <c r="F39" s="3"/>
       <c r="G39" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H39" s="3"/>
-      <c r="I39" s="11"/>
+      <c r="I39" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -3665,10 +3684,10 @@
         <v>20</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>118</v>
+        <v>22</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>8</v>
@@ -3700,13 +3719,13 @@
         <v>1</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>118</v>
+        <v>22</v>
       </c>
       <c r="I3" s="3" t="n">
         <v>8</v>
@@ -3723,7 +3742,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="n">
         <v>1</v>
@@ -3742,7 +3761,7 @@
         <v>20</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>29</v>
@@ -3762,7 +3781,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B5" s="3" t="n">
         <v>1</v>
@@ -3777,7 +3796,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>8</v>
@@ -3794,7 +3813,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B6" s="3" t="n">
         <v>1</v>
@@ -3809,7 +3828,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>8</v>
@@ -3826,7 +3845,7 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B7" s="3" t="n">
         <v>1</v>
@@ -3842,13 +3861,13 @@
         <v>1</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>8</v>
@@ -3865,7 +3884,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B8" s="3" t="n">
         <v>1</v>
@@ -3880,7 +3899,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>8</v>
@@ -3897,7 +3916,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B9" s="3" t="n">
         <v>1</v>
@@ -3913,13 +3932,13 @@
         <v>1</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>8</v>
@@ -3936,7 +3955,7 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B10" s="3" t="n">
         <v>1</v>
@@ -3951,10 +3970,10 @@
         <v>1</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>27</v>
@@ -3974,7 +3993,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B11" s="3" t="n">
         <v>0</v>
@@ -3990,7 +4009,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>8</v>
@@ -4007,7 +4026,7 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B12" s="3" t="n">
         <v>1</v>
@@ -4022,13 +4041,13 @@
         <v>1</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>8</v>
@@ -4045,7 +4064,7 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B13" s="3" t="n">
         <v>1</v>
@@ -4060,7 +4079,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>8</v>
@@ -4077,7 +4096,7 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B14" s="3" t="n">
         <v>1</v>
@@ -4093,7 +4112,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>8</v>
@@ -4110,7 +4129,7 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B15" s="3" t="n">
         <v>1</v>
@@ -4126,7 +4145,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>8</v>
@@ -4143,7 +4162,7 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B16" s="3" t="n">
         <v>1</v>
@@ -4158,7 +4177,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>8</v>
@@ -4175,7 +4194,7 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B17" s="3" t="n">
         <v>1</v>
@@ -4190,7 +4209,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>8</v>
@@ -4207,7 +4226,7 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B18" s="3" t="n">
         <v>1</v>
@@ -4225,10 +4244,10 @@
         <v>20</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>8</v>
@@ -4245,7 +4264,7 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B19" s="3" t="n">
         <v>1</v>
@@ -4261,7 +4280,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>8</v>
@@ -4278,7 +4297,7 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B20" s="3" t="n">
         <v>1</v>
@@ -4294,13 +4313,13 @@
         <v>1</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>8</v>
@@ -4317,7 +4336,7 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B21" s="3" t="n">
         <v>0</v>
@@ -4333,7 +4352,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>8</v>
@@ -4350,7 +4369,7 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B22" s="3" t="n">
         <v>1</v>
@@ -4365,7 +4384,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>8</v>
@@ -4382,7 +4401,7 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B23" s="3" t="n">
         <v>0</v>
@@ -4398,7 +4417,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>8</v>
@@ -4415,7 +4434,7 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B24" s="3" t="n">
         <v>1</v>
@@ -4431,7 +4450,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>8</v>
@@ -4448,7 +4467,7 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B25" s="3" t="n">
         <v>1</v>
@@ -4463,7 +4482,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>8</v>
@@ -4480,7 +4499,7 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B26" s="3" t="n">
         <v>1</v>
@@ -4495,7 +4514,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>8</v>
@@ -4512,7 +4531,7 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B27" s="3" t="n">
         <v>1</v>
@@ -4528,7 +4547,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>8</v>
@@ -4545,7 +4564,7 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B28" s="3" t="n">
         <v>1</v>
@@ -4560,7 +4579,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>8</v>
@@ -4577,7 +4596,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B29" s="3" t="n">
         <v>1</v>
@@ -4593,13 +4612,13 @@
         <v>1</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>8</v>
@@ -4616,7 +4635,7 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B30" s="3" t="n">
         <v>0</v>
@@ -4632,7 +4651,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>8</v>
@@ -4649,7 +4668,7 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B31" s="3" t="n">
         <v>0</v>
@@ -4665,7 +4684,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>8</v>
@@ -4682,7 +4701,7 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B32" s="3" t="n">
         <v>1</v>
@@ -4697,13 +4716,13 @@
         <v>1</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>8</v>
@@ -4720,7 +4739,7 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B33" s="3" t="n">
         <v>1</v>
@@ -4736,7 +4755,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I33" s="3" t="n">
         <v>8</v>
@@ -4753,7 +4772,7 @@
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B34" s="3" t="n">
         <v>1</v>
@@ -4769,7 +4788,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>8</v>
@@ -4786,7 +4805,7 @@
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B35" s="3" t="n">
         <v>1</v>
@@ -4801,13 +4820,13 @@
         <v>1</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G35" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="I35" s="3" t="n">
         <v>8</v>
@@ -4824,7 +4843,7 @@
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B36" s="3" t="n">
         <v>1</v>
@@ -4839,7 +4858,7 @@
         <v>0</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>8</v>
@@ -4856,7 +4875,7 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B37" s="3" t="n">
         <v>1</v>
@@ -4872,7 +4891,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>8</v>
@@ -4889,7 +4908,7 @@
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B38" s="3" t="n">
         <v>1</v>
@@ -4904,7 +4923,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>8</v>
@@ -4921,7 +4940,7 @@
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B39" s="3" t="n">
         <v>1</v>
@@ -4940,10 +4959,10 @@
         <v>131</v>
       </c>
       <c r="G39" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>8</v>
@@ -4960,7 +4979,7 @@
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B40" s="3" t="n">
         <v>0</v>
@@ -4976,7 +4995,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>8</v>
@@ -5008,13 +5027,13 @@
         <v>1</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="G41" s="3" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>118</v>
+        <v>22</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>8</v>
@@ -5046,13 +5065,13 @@
         <v>1</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G42" s="3" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="I42" s="3" t="n">
         <v>8</v>
@@ -5152,10 +5171,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>19</v>
@@ -5177,7 +5196,7 @@
         <v>20</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>29</v>
@@ -5201,10 +5220,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="C3" s="4" t="s">
         <v>19</v>
@@ -5222,7 +5241,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K3" s="3" t="n">
         <v>8</v>
@@ -5240,10 +5259,10 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>19</v>
@@ -5261,7 +5280,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>8</v>
@@ -5279,10 +5298,10 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>19</v>
@@ -5301,13 +5320,13 @@
         <v>1</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="K5" s="3" t="n">
         <v>8</v>
@@ -5328,10 +5347,10 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>19</v>
@@ -5349,7 +5368,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>8</v>
@@ -5367,10 +5386,10 @@
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>19</v>
@@ -5389,13 +5408,13 @@
         <v>1</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>8</v>
@@ -5416,10 +5435,10 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>19</v>
@@ -5437,10 +5456,10 @@
         <v>1</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>27</v>
@@ -5464,10 +5483,10 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>19</v>
@@ -5486,7 +5505,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>8</v>
@@ -5504,10 +5523,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>19</v>
@@ -5525,13 +5544,13 @@
         <v>1</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="K10" s="3" t="n">
         <v>8</v>
@@ -5552,10 +5571,10 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>19</v>
@@ -5573,7 +5592,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>8</v>
@@ -5591,10 +5610,10 @@
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>19</v>
@@ -5613,7 +5632,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K12" s="3" t="n">
         <v>8</v>
@@ -5631,10 +5650,10 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>19</v>
@@ -5653,7 +5672,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K13" s="3" t="n">
         <v>8</v>
@@ -5671,10 +5690,10 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>19</v>
@@ -5692,7 +5711,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K14" s="3" t="n">
         <v>8</v>
@@ -5710,10 +5729,10 @@
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>19</v>
@@ -5731,7 +5750,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K15" s="3" t="n">
         <v>8</v>
@@ -5749,10 +5768,10 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>19</v>
@@ -5773,10 +5792,10 @@
         <v>20</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="K16" s="3" t="n">
         <v>8</v>
@@ -5797,10 +5816,10 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>19</v>
@@ -5819,7 +5838,7 @@
         <v>0</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K17" s="3" t="n">
         <v>8</v>
@@ -5837,10 +5856,10 @@
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>19</v>
@@ -5859,13 +5878,13 @@
         <v>1</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="K18" s="3" t="n">
         <v>8</v>
@@ -5886,10 +5905,10 @@
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>19</v>
@@ -5908,7 +5927,7 @@
         <v>0</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K19" s="3" t="n">
         <v>8</v>
@@ -5926,10 +5945,10 @@
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>19</v>
@@ -5947,7 +5966,7 @@
         <v>0</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K20" s="3" t="n">
         <v>8</v>
@@ -5965,10 +5984,10 @@
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>19</v>
@@ -5987,7 +6006,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K21" s="3" t="n">
         <v>8</v>
@@ -6005,10 +6024,10 @@
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>19</v>
@@ -6027,7 +6046,7 @@
         <v>0</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K22" s="3" t="n">
         <v>8</v>
@@ -6045,10 +6064,10 @@
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>19</v>
@@ -6066,7 +6085,7 @@
         <v>0</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K23" s="3" t="n">
         <v>8</v>
@@ -6084,10 +6103,10 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>19</v>
@@ -6105,7 +6124,7 @@
         <v>0</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K24" s="3" t="n">
         <v>8</v>
@@ -6123,10 +6142,10 @@
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>19</v>
@@ -6145,7 +6164,7 @@
         <v>0</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K25" s="3" t="n">
         <v>8</v>
@@ -6163,10 +6182,10 @@
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>19</v>
@@ -6184,7 +6203,7 @@
         <v>0</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K26" s="3" t="n">
         <v>8</v>
@@ -6202,10 +6221,10 @@
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>19</v>
@@ -6224,13 +6243,13 @@
         <v>1</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="K27" s="3" t="n">
         <v>8</v>
@@ -6251,10 +6270,10 @@
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>19</v>
@@ -6273,7 +6292,7 @@
         <v>0</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K28" s="3" t="n">
         <v>8</v>
@@ -6291,10 +6310,10 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>19</v>
@@ -6313,7 +6332,7 @@
         <v>0</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K29" s="3" t="n">
         <v>8</v>
@@ -6331,10 +6350,10 @@
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>19</v>
@@ -6352,13 +6371,13 @@
         <v>1</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>8</v>
@@ -6379,10 +6398,10 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>19</v>
@@ -6401,7 +6420,7 @@
         <v>0</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K31" s="3" t="n">
         <v>8</v>
@@ -6419,10 +6438,10 @@
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>19</v>
@@ -6441,7 +6460,7 @@
         <v>0</v>
       </c>
       <c r="I32" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K32" s="3" t="n">
         <v>8</v>
@@ -6459,10 +6478,10 @@
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>19</v>
@@ -6480,13 +6499,13 @@
         <v>1</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="K33" s="3" t="n">
         <v>8</v>
@@ -6507,10 +6526,10 @@
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>19</v>
@@ -6528,7 +6547,7 @@
         <v>0</v>
       </c>
       <c r="I34" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K34" s="3" t="n">
         <v>8</v>
@@ -6546,10 +6565,10 @@
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>19</v>
@@ -6568,7 +6587,7 @@
         <v>0</v>
       </c>
       <c r="I35" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K35" s="3" t="n">
         <v>8</v>
@@ -6586,10 +6605,10 @@
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>19</v>
@@ -6607,7 +6626,7 @@
         <v>0</v>
       </c>
       <c r="I36" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K36" s="3" t="n">
         <v>8</v>
@@ -6625,10 +6644,10 @@
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="3" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C37" s="4" t="s">
         <v>19</v>
@@ -6647,13 +6666,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>8</v>
@@ -6671,10 +6690,10 @@
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C38" s="4" t="s">
         <v>19</v>
@@ -6693,7 +6712,7 @@
         <v>0</v>
       </c>
       <c r="I38" s="3" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="K38" s="3" t="n">
         <v>8</v>
@@ -6711,13 +6730,13 @@
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D39" s="3" t="n">
         <v>1</v>
@@ -6732,13 +6751,13 @@
         <v>1</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>118</v>
+        <v>22</v>
       </c>
       <c r="K39" s="3" t="n">
         <v>8</v>
@@ -6756,14 +6775,14 @@
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B40" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C40" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>115</v>
-      </c>
       <c r="D40" s="3" t="n">
         <v>1</v>
       </c>
@@ -6777,13 +6796,13 @@
         <v>1</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="K40" s="3" t="n">
         <v>8</v>
@@ -6801,13 +6820,13 @@
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>122</v>
+        <v>17</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>123</v>
+        <v>18</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D41" s="4" t="n">
         <v>1</v>
@@ -6825,10 +6844,10 @@
         <v>20</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>118</v>
+        <v>22</v>
       </c>
       <c r="K41" s="3" t="n">
         <v>8</v>
@@ -6846,13 +6865,13 @@
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>122</v>
+        <v>17</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>124</v>
+        <v>23</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D42" s="4" t="n">
         <v>1</v>
@@ -6867,13 +6886,13 @@
         <v>1</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>117</v>
+        <v>21</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>118</v>
+        <v>22</v>
       </c>
       <c r="K42" s="3" t="n">
         <v>8</v>

</xml_diff>

<commit_message>
* Removed: Integration error * Added: Pyramidal cells
</commit_message>
<xml_diff>
--- a/parameters/neurons_parameters.xlsx
+++ b/parameters/neurons_parameters.xlsx
@@ -791,6 +791,9 @@
         <v>0</v>
       </c>
       <c r="O2" s="3"/>
+      <c r="P2" s="0" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
@@ -836,6 +839,9 @@
         <v>0</v>
       </c>
       <c r="O3" s="3"/>
+      <c r="P3" s="0" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">

</xml_diff>

<commit_message>
Work on running full local model. Fit Delta eta in min max range.
</commit_message>
<xml_diff>
--- a/parameters/neurons_parameters.xlsx
+++ b/parameters/neurons_parameters.xlsx
@@ -784,7 +784,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q44"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="11.62"/>
@@ -2689,8 +2689,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Обычный"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -2701,7 +2701,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:U127"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="49.77"/>
@@ -2812,8 +2812,8 @@
       <c r="K2" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L2" s="2" t="n">
-        <v>85</v>
+      <c r="L2" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M2" s="8" t="n">
         <v>5</v>
@@ -2874,8 +2874,8 @@
       <c r="K3" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L3" s="2" t="n">
-        <v>40</v>
+      <c r="L3" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M3" s="8" t="n">
         <v>5</v>
@@ -2936,8 +2936,8 @@
       <c r="K4" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L4" s="2" t="n">
-        <v>110</v>
+      <c r="L4" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M4" s="8" t="n">
         <v>5</v>
@@ -2998,8 +2998,8 @@
       <c r="K5" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L5" s="2" t="n">
-        <v>65</v>
+      <c r="L5" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M5" s="8" t="n">
         <v>5</v>
@@ -3060,8 +3060,8 @@
       <c r="K6" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L6" s="2" t="n">
-        <v>100</v>
+      <c r="L6" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M6" s="8" t="n">
         <v>5</v>
@@ -3122,8 +3122,8 @@
       <c r="K7" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L7" s="2" t="n">
-        <v>90</v>
+      <c r="L7" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M7" s="8" t="n">
         <v>5</v>
@@ -3184,8 +3184,8 @@
       <c r="K8" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L8" s="2" t="n">
-        <v>20</v>
+      <c r="L8" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M8" s="8" t="n">
         <v>5</v>
@@ -3246,8 +3246,8 @@
       <c r="K9" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L9" s="2" t="n">
-        <v>55</v>
+      <c r="L9" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M9" s="8" t="n">
         <v>5</v>
@@ -3308,8 +3308,8 @@
       <c r="K10" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L10" s="2" t="n">
-        <v>60</v>
+      <c r="L10" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M10" s="8" t="n">
         <v>5</v>
@@ -3370,8 +3370,8 @@
       <c r="K11" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L11" s="2" t="n">
-        <v>45</v>
+      <c r="L11" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M11" s="8" t="n">
         <v>5</v>
@@ -3432,8 +3432,8 @@
       <c r="K12" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L12" s="2" t="n">
-        <v>105</v>
+      <c r="L12" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M12" s="8" t="n">
         <v>5</v>
@@ -3494,8 +3494,8 @@
       <c r="K13" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L13" s="2" t="n">
-        <v>15</v>
+      <c r="L13" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M13" s="8" t="n">
         <v>5</v>
@@ -3556,8 +3556,8 @@
       <c r="K14" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L14" s="2" t="n">
-        <v>95</v>
+      <c r="L14" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M14" s="8" t="n">
         <v>5</v>
@@ -3618,8 +3618,8 @@
       <c r="K15" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L15" s="2" t="n">
-        <v>35</v>
+      <c r="L15" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M15" s="8" t="n">
         <v>5</v>
@@ -3680,8 +3680,8 @@
       <c r="K16" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L16" s="2" t="n">
-        <v>50</v>
+      <c r="L16" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M16" s="8" t="n">
         <v>5</v>
@@ -3742,8 +3742,8 @@
       <c r="K17" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L17" s="2" t="n">
-        <v>30</v>
+      <c r="L17" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M17" s="8" t="n">
         <v>5</v>
@@ -3804,8 +3804,8 @@
       <c r="K18" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L18" s="2" t="n">
-        <v>80</v>
+      <c r="L18" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M18" s="8" t="n">
         <v>5</v>
@@ -3866,8 +3866,8 @@
       <c r="K19" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L19" s="2" t="n">
-        <v>70</v>
+      <c r="L19" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M19" s="8" t="n">
         <v>5</v>
@@ -3928,8 +3928,8 @@
       <c r="K20" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L20" s="2" t="n">
-        <v>75</v>
+      <c r="L20" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M20" s="8" t="n">
         <v>5</v>
@@ -3990,8 +3990,8 @@
       <c r="K21" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="L21" s="2" t="n">
-        <v>25</v>
+      <c r="L21" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M21" s="8" t="n">
         <v>5</v>
@@ -4052,8 +4052,8 @@
       <c r="K22" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L22" s="2" t="n">
-        <v>67</v>
+      <c r="L22" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M22" s="8" t="n">
         <v>5</v>
@@ -4114,8 +4114,8 @@
       <c r="K23" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L23" s="2" t="n">
-        <v>47</v>
+      <c r="L23" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M23" s="8" t="n">
         <v>5</v>
@@ -4176,8 +4176,8 @@
       <c r="K24" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L24" s="2" t="n">
-        <v>72</v>
+      <c r="L24" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M24" s="8" t="n">
         <v>5</v>
@@ -4238,8 +4238,8 @@
       <c r="K25" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L25" s="2" t="n">
-        <v>97</v>
+      <c r="L25" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M25" s="8" t="n">
         <v>5</v>
@@ -4300,8 +4300,8 @@
       <c r="K26" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L26" s="2" t="n">
-        <v>77</v>
+      <c r="L26" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M26" s="8" t="n">
         <v>5</v>
@@ -4362,8 +4362,8 @@
       <c r="K27" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L27" s="2" t="n">
-        <v>87</v>
+      <c r="L27" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M27" s="8" t="n">
         <v>5</v>
@@ -4424,8 +4424,8 @@
       <c r="K28" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L28" s="2" t="n">
-        <v>32</v>
+      <c r="L28" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M28" s="8" t="n">
         <v>5</v>
@@ -4486,8 +4486,8 @@
       <c r="K29" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L29" s="2" t="n">
-        <v>102</v>
+      <c r="L29" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M29" s="8" t="n">
         <v>5</v>
@@ -4548,8 +4548,8 @@
       <c r="K30" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L30" s="2" t="n">
-        <v>42</v>
+      <c r="L30" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M30" s="8" t="n">
         <v>5</v>
@@ -4610,8 +4610,8 @@
       <c r="K31" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L31" s="2" t="n">
-        <v>57</v>
+      <c r="L31" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M31" s="8" t="n">
         <v>5</v>
@@ -4672,8 +4672,8 @@
       <c r="K32" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L32" s="2" t="n">
-        <v>27</v>
+      <c r="L32" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M32" s="8" t="n">
         <v>5</v>
@@ -4734,8 +4734,8 @@
       <c r="K33" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L33" s="2" t="n">
-        <v>17</v>
+      <c r="L33" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M33" s="8" t="n">
         <v>5</v>
@@ -4796,8 +4796,8 @@
       <c r="K34" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L34" s="2" t="n">
-        <v>92</v>
+      <c r="L34" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M34" s="8" t="n">
         <v>5</v>
@@ -4858,8 +4858,8 @@
       <c r="K35" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L35" s="2" t="n">
-        <v>22</v>
+      <c r="L35" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M35" s="8" t="n">
         <v>5</v>
@@ -4920,8 +4920,8 @@
       <c r="K36" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L36" s="2" t="n">
-        <v>62</v>
+      <c r="L36" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M36" s="8" t="n">
         <v>5</v>
@@ -4982,8 +4982,8 @@
       <c r="K37" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L37" s="2" t="n">
-        <v>107</v>
+      <c r="L37" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M37" s="8" t="n">
         <v>5</v>
@@ -5044,8 +5044,8 @@
       <c r="K38" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L38" s="2" t="n">
-        <v>12</v>
+      <c r="L38" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M38" s="8" t="n">
         <v>5</v>
@@ -5106,8 +5106,8 @@
       <c r="K39" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L39" s="2" t="n">
-        <v>82</v>
+      <c r="L39" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M39" s="8" t="n">
         <v>5</v>
@@ -5168,8 +5168,8 @@
       <c r="K40" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L40" s="2" t="n">
-        <v>37</v>
+      <c r="L40" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M40" s="8" t="n">
         <v>5</v>
@@ -5230,8 +5230,8 @@
       <c r="K41" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="L41" s="2" t="n">
-        <v>52</v>
+      <c r="L41" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M41" s="8" t="n">
         <v>5</v>
@@ -5643,7 +5643,7 @@
       <c r="K49" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L49" s="4" t="n">
+      <c r="L49" s="3" t="n">
         <v>-100000</v>
       </c>
       <c r="M49" s="4" t="n">
@@ -6025,7 +6025,7 @@
       <c r="K57" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L57" s="4" t="n">
+      <c r="L57" s="3" t="n">
         <v>-100000</v>
       </c>
       <c r="M57" s="4" t="n">
@@ -6831,7 +6831,7 @@
       <c r="K74" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="L74" s="4" t="n">
+      <c r="L74" s="3" t="n">
         <v>-100000</v>
       </c>
       <c r="M74" s="4" t="n">
@@ -7073,8 +7073,8 @@
       <c r="K79" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L79" s="13" t="n">
-        <v>5</v>
+      <c r="L79" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M79" s="13" t="n">
         <v>5</v>
@@ -7118,8 +7118,8 @@
       <c r="K80" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L80" s="13" t="n">
-        <v>10</v>
+      <c r="L80" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M80" s="13" t="n">
         <v>5</v>
@@ -7163,8 +7163,8 @@
       <c r="K81" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L81" s="13" t="n">
-        <v>15</v>
+      <c r="L81" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M81" s="13" t="n">
         <v>5</v>
@@ -7208,8 +7208,8 @@
       <c r="K82" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L82" s="13" t="n">
-        <v>20</v>
+      <c r="L82" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M82" s="13" t="n">
         <v>5</v>
@@ -7253,8 +7253,8 @@
       <c r="K83" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L83" s="13" t="n">
-        <v>25</v>
+      <c r="L83" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M83" s="13" t="n">
         <v>5</v>
@@ -7298,8 +7298,8 @@
       <c r="K84" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L84" s="13" t="n">
-        <v>30</v>
+      <c r="L84" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M84" s="13" t="n">
         <v>5</v>
@@ -7343,8 +7343,8 @@
       <c r="K85" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L85" s="13" t="n">
-        <v>35</v>
+      <c r="L85" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M85" s="13" t="n">
         <v>5</v>
@@ -7388,8 +7388,8 @@
       <c r="K86" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L86" s="13" t="n">
-        <v>40</v>
+      <c r="L86" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M86" s="13" t="n">
         <v>5</v>
@@ -7433,8 +7433,8 @@
       <c r="K87" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L87" s="13" t="n">
-        <v>45</v>
+      <c r="L87" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M87" s="13" t="n">
         <v>5</v>
@@ -7478,8 +7478,8 @@
       <c r="K88" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L88" s="13" t="n">
-        <v>50</v>
+      <c r="L88" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M88" s="13" t="n">
         <v>5</v>
@@ -7523,8 +7523,8 @@
       <c r="K89" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L89" s="13" t="n">
-        <v>55</v>
+      <c r="L89" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M89" s="13" t="n">
         <v>5</v>
@@ -7568,8 +7568,8 @@
       <c r="K90" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L90" s="13" t="n">
-        <v>60</v>
+      <c r="L90" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M90" s="13" t="n">
         <v>5</v>
@@ -7613,8 +7613,8 @@
       <c r="K91" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L91" s="13" t="n">
-        <v>65</v>
+      <c r="L91" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M91" s="13" t="n">
         <v>5</v>
@@ -7658,8 +7658,8 @@
       <c r="K92" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L92" s="13" t="n">
-        <v>70</v>
+      <c r="L92" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M92" s="13" t="n">
         <v>5</v>
@@ -7703,8 +7703,8 @@
       <c r="K93" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L93" s="13" t="n">
-        <v>75</v>
+      <c r="L93" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M93" s="13" t="n">
         <v>5</v>
@@ -7748,8 +7748,8 @@
       <c r="K94" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L94" s="13" t="n">
-        <v>80</v>
+      <c r="L94" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M94" s="13" t="n">
         <v>5</v>
@@ -7793,8 +7793,8 @@
       <c r="K95" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L95" s="13" t="n">
-        <v>85</v>
+      <c r="L95" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M95" s="13" t="n">
         <v>5</v>
@@ -7838,8 +7838,8 @@
       <c r="K96" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L96" s="13" t="n">
-        <v>90</v>
+      <c r="L96" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M96" s="13" t="n">
         <v>5</v>
@@ -7883,8 +7883,8 @@
       <c r="K97" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L97" s="13" t="n">
-        <v>95</v>
+      <c r="L97" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M97" s="13" t="n">
         <v>5</v>
@@ -7928,8 +7928,8 @@
       <c r="K98" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L98" s="13" t="n">
-        <v>100</v>
+      <c r="L98" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M98" s="13" t="n">
         <v>5</v>
@@ -7973,8 +7973,8 @@
       <c r="K99" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L99" s="13" t="n">
-        <v>105</v>
+      <c r="L99" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M99" s="13" t="n">
         <v>5</v>
@@ -8018,8 +8018,8 @@
       <c r="K100" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L100" s="13" t="n">
-        <v>110</v>
+      <c r="L100" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M100" s="13" t="n">
         <v>5</v>
@@ -8063,8 +8063,8 @@
       <c r="K101" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L101" s="13" t="n">
-        <v>115</v>
+      <c r="L101" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M101" s="13" t="n">
         <v>5</v>
@@ -8108,8 +8108,8 @@
       <c r="K102" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="L102" s="13" t="n">
-        <v>120</v>
+      <c r="L102" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M102" s="13" t="n">
         <v>5</v>
@@ -8153,8 +8153,8 @@
       <c r="K103" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L103" s="14" t="n">
-        <v>5</v>
+      <c r="L103" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M103" s="13" t="n">
         <v>5</v>
@@ -8198,8 +8198,8 @@
       <c r="K104" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L104" s="14" t="n">
-        <v>10</v>
+      <c r="L104" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M104" s="13" t="n">
         <v>5</v>
@@ -8242,8 +8242,8 @@
       <c r="K105" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L105" s="14" t="n">
-        <v>15</v>
+      <c r="L105" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M105" s="13" t="n">
         <v>5</v>
@@ -8286,8 +8286,8 @@
       <c r="K106" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L106" s="14" t="n">
-        <v>20</v>
+      <c r="L106" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M106" s="13" t="n">
         <v>5</v>
@@ -8330,8 +8330,8 @@
       <c r="K107" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L107" s="14" t="n">
-        <v>25</v>
+      <c r="L107" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M107" s="13" t="n">
         <v>5</v>
@@ -8374,8 +8374,8 @@
       <c r="K108" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L108" s="14" t="n">
-        <v>30</v>
+      <c r="L108" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M108" s="13" t="n">
         <v>5</v>
@@ -8418,8 +8418,8 @@
       <c r="K109" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L109" s="14" t="n">
-        <v>35</v>
+      <c r="L109" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M109" s="13" t="n">
         <v>5</v>
@@ -8462,8 +8462,8 @@
       <c r="K110" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L110" s="14" t="n">
-        <v>40</v>
+      <c r="L110" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M110" s="13" t="n">
         <v>5</v>
@@ -8506,8 +8506,8 @@
       <c r="K111" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L111" s="14" t="n">
-        <v>45</v>
+      <c r="L111" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M111" s="13" t="n">
         <v>5</v>
@@ -8550,8 +8550,8 @@
       <c r="K112" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L112" s="14" t="n">
-        <v>50</v>
+      <c r="L112" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M112" s="13" t="n">
         <v>5</v>
@@ -8594,8 +8594,8 @@
       <c r="K113" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L113" s="14" t="n">
-        <v>55</v>
+      <c r="L113" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M113" s="13" t="n">
         <v>5</v>
@@ -8638,8 +8638,8 @@
       <c r="K114" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L114" s="14" t="n">
-        <v>60</v>
+      <c r="L114" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M114" s="13" t="n">
         <v>5</v>
@@ -8682,8 +8682,8 @@
       <c r="K115" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L115" s="14" t="n">
-        <v>65</v>
+      <c r="L115" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M115" s="13" t="n">
         <v>5</v>
@@ -8726,8 +8726,8 @@
       <c r="K116" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L116" s="14" t="n">
-        <v>70</v>
+      <c r="L116" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M116" s="13" t="n">
         <v>5</v>
@@ -8770,8 +8770,8 @@
       <c r="K117" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L117" s="14" t="n">
-        <v>75</v>
+      <c r="L117" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M117" s="13" t="n">
         <v>5</v>
@@ -8814,8 +8814,8 @@
       <c r="K118" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L118" s="14" t="n">
-        <v>80</v>
+      <c r="L118" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M118" s="13" t="n">
         <v>5</v>
@@ -8858,8 +8858,8 @@
       <c r="K119" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L119" s="14" t="n">
-        <v>85</v>
+      <c r="L119" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M119" s="13" t="n">
         <v>5</v>
@@ -8903,8 +8903,8 @@
       <c r="K120" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L120" s="14" t="n">
-        <v>90</v>
+      <c r="L120" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M120" s="13" t="n">
         <v>5</v>
@@ -8947,8 +8947,8 @@
       <c r="K121" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L121" s="14" t="n">
-        <v>95</v>
+      <c r="L121" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M121" s="13" t="n">
         <v>5</v>
@@ -8991,8 +8991,8 @@
       <c r="K122" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L122" s="14" t="n">
-        <v>100</v>
+      <c r="L122" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M122" s="13" t="n">
         <v>5</v>
@@ -9035,8 +9035,8 @@
       <c r="K123" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L123" s="14" t="n">
-        <v>105</v>
+      <c r="L123" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M123" s="13" t="n">
         <v>5</v>
@@ -9079,8 +9079,8 @@
       <c r="K124" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L124" s="14" t="n">
-        <v>110</v>
+      <c r="L124" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M124" s="13" t="n">
         <v>5</v>
@@ -9123,8 +9123,8 @@
       <c r="K125" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L125" s="14" t="n">
-        <v>115</v>
+      <c r="L125" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M125" s="13" t="n">
         <v>5</v>
@@ -9167,8 +9167,8 @@
       <c r="K126" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="L126" s="14" t="n">
-        <v>120</v>
+      <c r="L126" s="3" t="n">
+        <v>-100000</v>
       </c>
       <c r="M126" s="13" t="n">
         <v>5</v>
@@ -9193,8 +9193,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Обычный"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Page &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -9205,7 +9205,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="11.62"/>
@@ -10686,8 +10686,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Обычный"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Страница &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Страница &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
@@ -10698,7 +10698,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q42"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="3" width="41.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="3" width="26.64"/>
@@ -12508,8 +12508,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Обычный"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Обычный"&amp;12Страница &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Страница &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>